<commit_message>
update: reports updated as of march 3-10 2026
</commit_message>
<xml_diff>
--- a/reports/Angola_1.1_trade_balance_2003-2025.xlsx
+++ b/reports/Angola_1.1_trade_balance_2003-2025.xlsx
@@ -558,10 +558,10 @@
         <v>13753197951.671</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -599,10 +599,10 @@
         <v>19449718096.978</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>0.7598721598078365</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>1.037485140215486</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -640,10 +640,10 @@
         <v>29853580609.199</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>1.018159383974958</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>1.071619132840016</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -681,10 +681,10 @@
         <v>42684001130.593</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>0.9964198023491659</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>0.9936473336433598</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -722,10 +722,10 @@
         <v>54374326930.998</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>0.8762011070012461</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>1.059117332682969</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -763,10 +763,10 @@
         <v>88202394131.57501</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>1.169797356503398</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>0.9708288531140793</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -804,10 +804,10 @@
         <v>57774834915.186</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>1.340895850688063</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>1.017591329991285</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -845,10 +845,10 @@
         <v>69330714961.562</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>1.14325910578991</v>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>0.984122582880648</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -886,10 +886,10 @@
         <v>84533037403.558</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>1.134542472086246</v>
       </c>
       <c r="M10">
-        <v>1</v>
+        <v>1.003319832857205</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -927,10 +927,10 @@
         <v>97602647040.14799</v>
       </c>
       <c r="L11">
-        <v>1</v>
+        <v>1.29889876466322</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>0.9387166857837813</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -968,10 +968,10 @@
         <v>96752864734.39801</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>1.094487920684857</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>0.9364630532973149</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1009,10 +1009,10 @@
         <v>93108204542.412</v>
       </c>
       <c r="L13">
-        <v>1</v>
+        <v>1.012063636667582</v>
       </c>
       <c r="M13">
-        <v>1</v>
+        <v>0.9068730861746349</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1050,10 +1050,10 @@
         <v>55366337680.442</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>1.163072052808997</v>
       </c>
       <c r="M14">
-        <v>1</v>
+        <v>0.9209108448602463</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1091,10 +1091,10 @@
         <v>39963222663.098</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>1.230960215939978</v>
       </c>
       <c r="M15">
-        <v>1</v>
+        <v>0.9911678214462301</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1132,10 +1132,10 @@
         <v>48586367162.946</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>1.301844220990532</v>
       </c>
       <c r="M16">
-        <v>1</v>
+        <v>0.9508501503204908</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1173,10 +1173,10 @@
         <v>54540453118.876</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>1.546506247683954</v>
       </c>
       <c r="M17">
-        <v>1</v>
+        <v>0.9202227100799412</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1214,10 +1214,10 @@
         <v>46995627764.019</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>1.472369654202647</v>
       </c>
       <c r="M18">
-        <v>1</v>
+        <v>0.9445330135891916</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1255,10 +1255,10 @@
         <v>31559663691.815</v>
       </c>
       <c r="L19">
-        <v>1</v>
+        <v>1.227654674826444</v>
       </c>
       <c r="M19">
-        <v>1</v>
+        <v>0.9240671902293832</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1296,10 +1296,10 @@
         <v>42909650746.16</v>
       </c>
       <c r="L20">
-        <v>1</v>
+        <v>1.205642790257764</v>
       </c>
       <c r="M20">
-        <v>1</v>
+        <v>1.029893120475081</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1337,10 +1337,10 @@
         <v>67873491423.793</v>
       </c>
       <c r="L21">
-        <v>1</v>
+        <v>1.212498451158243</v>
       </c>
       <c r="M21">
-        <v>1</v>
+        <v>0.9639844945299021</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1378,10 +1378,10 @@
         <v>53211285059.012</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>1.201663089554985</v>
       </c>
       <c r="M22">
-        <v>1</v>
+        <v>0.9839671468180234</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1419,10 +1419,10 @@
         <v>50051223235.425</v>
       </c>
       <c r="L23">
-        <v>1</v>
+        <v>1.158966808266594</v>
       </c>
       <c r="M23">
-        <v>1</v>
+        <v>1.032409636557851</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1460,10 +1460,10 @@
         <v>4831976085.080999</v>
       </c>
       <c r="L24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M24">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>